<commit_message>
Revision(Minor): Section Management: Fixed bugs in filters, Changed adviserId from not null to null
</commit_message>
<xml_diff>
--- a/backend/edutrack/src/main/resources/templates/sf2-template.xlsx
+++ b/backend/edutrack/src/main/resources/templates/sf2-template.xlsx
@@ -3026,26 +3026,39 @@
     <col width="14.09765625" customWidth="1" style="204" min="3" max="3"/>
     <col width="17.296875" customWidth="1" style="204" min="4" max="4"/>
     <col width="0.09765625" customWidth="1" style="204" min="5" max="5"/>
-    <col width="0.8984375" customWidth="1" style="204" min="6" max="6"/>
-    <col width="2" customWidth="1" style="204" min="7" max="7"/>
-    <col width="2.8984375" customWidth="1" style="204" min="8" max="11"/>
-    <col width="2.59765625" customWidth="1" style="204" min="12" max="12"/>
-    <col width="0.296875" customWidth="1" style="204" min="13" max="13"/>
-    <col width="2.8984375" customWidth="1" style="204" min="14" max="17"/>
-    <col width="0.8984375" customWidth="1" style="204" min="18" max="18"/>
-    <col width="2" customWidth="1" style="204" min="19" max="19"/>
-    <col width="2.8984375" customWidth="1" style="204" min="20" max="21"/>
-    <col width="0.69921875" customWidth="1" style="204" min="22" max="22"/>
-    <col width="2.09765625" customWidth="1" style="204" min="23" max="23"/>
-    <col width="1.09765625" customWidth="1" style="204" min="24" max="24"/>
-    <col width="1.69921875" customWidth="1" style="204" min="25" max="26"/>
-    <col width="1.09765625" customWidth="1" style="204" min="27" max="27"/>
-    <col width="2.8984375" customWidth="1" style="204" min="28" max="32"/>
-    <col width="2.69921875" customWidth="1" style="204" min="33" max="33"/>
-    <col width="0.09765625" customWidth="1" style="204" min="34" max="34"/>
-    <col width="2.8984375" customWidth="1" style="204" min="35" max="36"/>
-    <col width="1.09765625" customWidth="1" style="204" min="37" max="37"/>
-    <col width="1.69921875" customWidth="1" style="204" min="38" max="39"/>
+    <col width="4.2" customWidth="1" style="204" min="6" max="6"/>
+    <col width="4.2" customWidth="1" style="204" min="7" max="7"/>
+    <col width="4.2" customWidth="1" style="204" min="8" max="11"/>
+    <col width="4.2" customWidth="1" style="204" min="9" max="9"/>
+    <col width="4.2" customWidth="1" style="204" min="10" max="10"/>
+    <col width="4.2" customWidth="1" style="204" min="11" max="11"/>
+    <col width="4.2" customWidth="1" style="204" min="12" max="12"/>
+    <col width="4.2" customWidth="1" style="204" min="13" max="13"/>
+    <col width="4.2" customWidth="1" style="204" min="14" max="17"/>
+    <col width="4.2" customWidth="1" style="204" min="15" max="15"/>
+    <col width="4.2" customWidth="1" style="204" min="16" max="16"/>
+    <col width="4.2" customWidth="1" style="204" min="17" max="17"/>
+    <col width="4.2" customWidth="1" style="204" min="18" max="18"/>
+    <col width="4.2" customWidth="1" style="204" min="19" max="19"/>
+    <col width="4.2" customWidth="1" style="204" min="20" max="21"/>
+    <col width="4.2" customWidth="1" style="204" min="21" max="21"/>
+    <col width="4.2" customWidth="1" style="204" min="22" max="22"/>
+    <col width="4.2" customWidth="1" style="204" min="23" max="23"/>
+    <col width="4.2" customWidth="1" style="204" min="24" max="24"/>
+    <col width="4.2" customWidth="1" style="204" min="25" max="26"/>
+    <col width="4.2" customWidth="1" style="204" min="26" max="26"/>
+    <col width="4.2" customWidth="1" style="204" min="27" max="27"/>
+    <col width="4.2" customWidth="1" style="204" min="28" max="32"/>
+    <col width="4.2" customWidth="1" style="204" min="29" max="29"/>
+    <col width="4.2" customWidth="1" style="204" min="30" max="30"/>
+    <col width="4.2" customWidth="1" style="204" min="31" max="31"/>
+    <col width="4.2" customWidth="1" style="204" min="32" max="32"/>
+    <col width="4.2" customWidth="1" style="204" min="33" max="33"/>
+    <col width="4.2" customWidth="1" style="204" min="34" max="34"/>
+    <col width="4.2" customWidth="1" style="204" min="35" max="36"/>
+    <col width="4.2" customWidth="1" style="204" min="36" max="36"/>
+    <col width="4.2" customWidth="1" style="204" min="37" max="37"/>
+    <col width="4.2" customWidth="1" style="204" min="38" max="39"/>
     <col width="5" customWidth="1" style="204" min="40" max="41"/>
     <col width="1.69921875" customWidth="1" style="204" min="42" max="42"/>
     <col width="10.09765625" customWidth="1" style="204" min="43" max="43"/>
@@ -3367,7 +3380,7 @@
       <c r="AJ8" s="9" t="n"/>
       <c r="AK8" s="253" t="n"/>
       <c r="AM8" s="254">
-        <f>COUNTIF(F8:AL8,"X")</f>
+        <f>COUNTIF(F8:AL8,"A")</f>
         <v/>
       </c>
       <c r="AN8" s="255" t="n"/>
@@ -3418,7 +3431,7 @@
       <c r="AJ9" s="9" t="n"/>
       <c r="AK9" s="21" t="n"/>
       <c r="AM9" s="254">
-        <f>COUNTIF(F9:AL9,"X")</f>
+        <f>COUNTIF(F9:AL9,"A")</f>
         <v/>
       </c>
       <c r="AN9" s="255" t="n"/>
@@ -3469,7 +3482,7 @@
       <c r="AJ10" s="9" t="n"/>
       <c r="AK10" s="21" t="n"/>
       <c r="AM10" s="254">
-        <f>COUNTIF(F10:AL10,"X")</f>
+        <f>COUNTIF(F10:AL10,"A")</f>
         <v/>
       </c>
       <c r="AN10" s="255" t="n"/>
@@ -3520,7 +3533,7 @@
       <c r="AJ11" s="9" t="n"/>
       <c r="AK11" s="21" t="n"/>
       <c r="AM11" s="254">
-        <f>COUNTIF(F11:AL11,"X")</f>
+        <f>COUNTIF(F11:AL11,"A")</f>
         <v/>
       </c>
       <c r="AN11" s="255" t="n"/>
@@ -3571,7 +3584,7 @@
       <c r="AJ12" s="9" t="n"/>
       <c r="AK12" s="21" t="n"/>
       <c r="AM12" s="254">
-        <f>COUNTIF(F12:AL12,"X")</f>
+        <f>COUNTIF(F12:AL12,"A")</f>
         <v/>
       </c>
       <c r="AN12" s="255" t="n"/>
@@ -3622,7 +3635,7 @@
       <c r="AJ13" s="9" t="n"/>
       <c r="AK13" s="21" t="n"/>
       <c r="AM13" s="254">
-        <f>COUNTIF(F13:AL13,"X")</f>
+        <f>COUNTIF(F13:AL13,"A")</f>
         <v/>
       </c>
       <c r="AN13" s="255" t="n"/>
@@ -3673,7 +3686,7 @@
       <c r="AJ14" s="9" t="n"/>
       <c r="AK14" s="21" t="n"/>
       <c r="AM14" s="254">
-        <f>COUNTIF(F14:AL14,"X")</f>
+        <f>COUNTIF(F14:AL14,"A")</f>
         <v/>
       </c>
       <c r="AN14" s="255" t="n"/>
@@ -3724,7 +3737,7 @@
       <c r="AJ15" s="9" t="n"/>
       <c r="AK15" s="21" t="n"/>
       <c r="AM15" s="254">
-        <f>COUNTIF(F15:AL15,"X")</f>
+        <f>COUNTIF(F15:AL15,"A")</f>
         <v/>
       </c>
       <c r="AN15" s="255" t="n"/>
@@ -3775,7 +3788,7 @@
       <c r="AJ16" s="9" t="n"/>
       <c r="AK16" s="21" t="n"/>
       <c r="AM16" s="254">
-        <f>COUNTIF(F16:AL16,"X")</f>
+        <f>COUNTIF(F16:AL16,"A")</f>
         <v/>
       </c>
       <c r="AN16" s="255" t="n"/>
@@ -3824,7 +3837,7 @@
       <c r="AJ17" s="9" t="n"/>
       <c r="AK17" s="21" t="n"/>
       <c r="AM17" s="254">
-        <f>COUNTIF(F17:AL17,"X")</f>
+        <f>COUNTIF(F17:AL17,"A")</f>
         <v/>
       </c>
       <c r="AN17" s="255" t="n"/>
@@ -3879,7 +3892,7 @@
       <c r="AJ18" s="9" t="n"/>
       <c r="AK18" s="21" t="n"/>
       <c r="AM18" s="254">
-        <f>COUNTIF(F18:AL18,"X")</f>
+        <f>COUNTIF(F18:AL18,"A")</f>
         <v/>
       </c>
       <c r="AN18" s="255" t="n"/>
@@ -3930,7 +3943,7 @@
       <c r="AJ19" s="9" t="n"/>
       <c r="AK19" s="21" t="n"/>
       <c r="AM19" s="254">
-        <f>COUNTIF(F19:AL19,"X")</f>
+        <f>COUNTIF(F19:AL19,"A")</f>
         <v/>
       </c>
       <c r="AN19" s="255" t="n"/>
@@ -3981,7 +3994,7 @@
       <c r="AJ20" s="9" t="n"/>
       <c r="AK20" s="21" t="n"/>
       <c r="AM20" s="254">
-        <f>COUNTIF(F20:AL20,"X")</f>
+        <f>COUNTIF(F20:AL20,"A")</f>
         <v/>
       </c>
       <c r="AN20" s="255" t="n"/>
@@ -4032,7 +4045,7 @@
       <c r="AJ21" s="9" t="n"/>
       <c r="AK21" s="21" t="n"/>
       <c r="AM21" s="254">
-        <f>COUNTIF(F21:AL21,"X")</f>
+        <f>COUNTIF(F21:AL21,"A")</f>
         <v/>
       </c>
       <c r="AN21" s="255" t="n"/>
@@ -4083,7 +4096,7 @@
       <c r="AJ22" s="9" t="n"/>
       <c r="AK22" s="21" t="n"/>
       <c r="AM22" s="254">
-        <f>COUNTIF(F22:AL22,"X")</f>
+        <f>COUNTIF(F22:AL22,"A")</f>
         <v/>
       </c>
       <c r="AN22" s="255" t="n"/>
@@ -4134,7 +4147,7 @@
       <c r="AJ23" s="9" t="n"/>
       <c r="AK23" s="21" t="n"/>
       <c r="AM23" s="254">
-        <f>COUNTIF(F23:AL23,"X")</f>
+        <f>COUNTIF(F23:AL23,"A")</f>
         <v/>
       </c>
       <c r="AN23" s="255" t="n"/>
@@ -4185,7 +4198,7 @@
       <c r="AJ24" s="9" t="n"/>
       <c r="AK24" s="21" t="n"/>
       <c r="AM24" s="254">
-        <f>COUNTIF(F24:AL24,"X")</f>
+        <f>COUNTIF(F24:AL24,"A")</f>
         <v/>
       </c>
       <c r="AN24" s="255" t="n"/>
@@ -4234,7 +4247,7 @@
       <c r="AJ25" s="36" t="n"/>
       <c r="AK25" s="21" t="n"/>
       <c r="AM25" s="254">
-        <f>COUNTIF(F25:AL25,"X")</f>
+        <f>COUNTIF(F25:AL25,"A")</f>
         <v/>
       </c>
       <c r="AN25" s="255" t="n"/>
@@ -4285,12 +4298,12 @@
       <c r="AJ26" s="9" t="n"/>
       <c r="AK26" s="179" t="n"/>
       <c r="AM26" s="254">
-        <f>COUNTIF(F26:AL26,"X")</f>
+        <f>COUNTIF(F26:AL26,"A")</f>
         <v/>
       </c>
       <c r="AN26" s="255" t="n"/>
       <c r="AO26" s="254">
-        <f>$AW$4-AM26</f>
+        <f>AW4-AM26</f>
         <v/>
       </c>
       <c r="AP26" s="255" t="n"/>
@@ -4336,12 +4349,12 @@
       <c r="AJ27" s="9" t="n"/>
       <c r="AK27" s="179" t="n"/>
       <c r="AM27" s="254">
-        <f>COUNTIF(F27:AL27,"X")</f>
+        <f>COUNTIF(F27:AL27,"A")</f>
         <v/>
       </c>
       <c r="AN27" s="255" t="n"/>
       <c r="AO27" s="254">
-        <f>$AW$4-AM27</f>
+        <f>AW4-AM27</f>
         <v/>
       </c>
       <c r="AP27" s="255" t="n"/>
@@ -4385,12 +4398,12 @@
       <c r="AJ28" s="9" t="n"/>
       <c r="AK28" s="21" t="n"/>
       <c r="AM28" s="254">
-        <f>COUNTIF(F28:AL28,"X")</f>
+        <f>COUNTIF(F28:AL28,"A")</f>
         <v/>
       </c>
       <c r="AN28" s="255" t="n"/>
       <c r="AO28" s="254">
-        <f>$AW$4-AM28</f>
+        <f>AW4-AM28</f>
         <v/>
       </c>
       <c r="AP28" s="255" t="n"/>
@@ -4434,12 +4447,12 @@
       <c r="AJ29" s="36" t="n"/>
       <c r="AK29" s="21" t="n"/>
       <c r="AM29" s="254">
-        <f>COUNTIF(F29:AL29,"X")</f>
+        <f>COUNTIF(F29:AL29,"A")</f>
         <v/>
       </c>
       <c r="AN29" s="255" t="n"/>
       <c r="AO29" s="254">
-        <f>$AW$4-AM29</f>
+        <f>AW4-AM29</f>
         <v/>
       </c>
       <c r="AP29" s="255" t="n"/>
@@ -4485,12 +4498,12 @@
       <c r="AJ30" s="9" t="n"/>
       <c r="AK30" s="179" t="n"/>
       <c r="AM30" s="254">
-        <f>COUNTIF(F30:AL30,"X")</f>
+        <f>COUNTIF(F30:AL30,"A")</f>
         <v/>
       </c>
       <c r="AN30" s="255" t="n"/>
       <c r="AO30" s="254">
-        <f>$AW$4-AM30</f>
+        <f>AW4-AM30</f>
         <v/>
       </c>
       <c r="AP30" s="255" t="n"/>
@@ -4535,9 +4548,15 @@
       <c r="AI31" s="55" t="n"/>
       <c r="AJ31" s="9" t="n"/>
       <c r="AK31" s="179" t="n"/>
-      <c r="AM31" s="254" t="n"/>
+      <c r="AM31" s="254">
+        <f>COUNTIF(F31:AL31,"A")</f>
+        <v/>
+      </c>
       <c r="AN31" s="255" t="n"/>
-      <c r="AO31" s="254" t="n"/>
+      <c r="AO31" s="254">
+        <f>AW4-AM31</f>
+        <v/>
+      </c>
       <c r="AP31" s="255" t="n"/>
       <c r="AQ31" s="48" t="n"/>
       <c r="AR31" s="220" t="n"/>
@@ -4578,9 +4597,15 @@
       <c r="AI32" s="55" t="n"/>
       <c r="AJ32" s="9" t="n"/>
       <c r="AK32" s="179" t="n"/>
-      <c r="AM32" s="254" t="n"/>
+      <c r="AM32" s="254">
+        <f>COUNTIF(F32:AL32,"A")</f>
+        <v/>
+      </c>
       <c r="AN32" s="255" t="n"/>
-      <c r="AO32" s="254" t="n"/>
+      <c r="AO32" s="254">
+        <f>AW4-AM32</f>
+        <v/>
+      </c>
       <c r="AP32" s="255" t="n"/>
       <c r="AQ32" s="48" t="n"/>
       <c r="AR32" s="220" t="n"/>
@@ -4673,7 +4698,7 @@
       <c r="AJ34" s="9" t="n"/>
       <c r="AK34" s="21" t="n"/>
       <c r="AM34" s="254">
-        <f>COUNTIF(F34:AL34,"X")</f>
+        <f>COUNTIF(F34:AL34,"A")</f>
         <v/>
       </c>
       <c r="AN34" s="255" t="n"/>
@@ -4722,7 +4747,7 @@
       <c r="AJ35" s="9" t="n"/>
       <c r="AK35" s="21" t="n"/>
       <c r="AM35" s="254">
-        <f>COUNTIF(F35:AL35,"X")</f>
+        <f>COUNTIF(F35:AL35,"A")</f>
         <v/>
       </c>
       <c r="AN35" s="255" t="n"/>
@@ -4771,7 +4796,7 @@
       <c r="AJ36" s="9" t="n"/>
       <c r="AK36" s="21" t="n"/>
       <c r="AM36" s="254">
-        <f>COUNTIF(F36:AL36,"X")</f>
+        <f>COUNTIF(F36:AL36,"A")</f>
         <v/>
       </c>
       <c r="AN36" s="255" t="n"/>
@@ -4820,7 +4845,7 @@
       <c r="AJ37" s="9" t="n"/>
       <c r="AK37" s="21" t="n"/>
       <c r="AM37" s="254">
-        <f>COUNTIF(F37:AL37,"X")</f>
+        <f>COUNTIF(F37:AL37,"A")</f>
         <v/>
       </c>
       <c r="AN37" s="255" t="n"/>
@@ -4869,7 +4894,7 @@
       <c r="AJ38" s="9" t="n"/>
       <c r="AK38" s="21" t="n"/>
       <c r="AM38" s="254">
-        <f>COUNTIF(F38:AL38,"X")</f>
+        <f>COUNTIF(F38:AL38,"A")</f>
         <v/>
       </c>
       <c r="AN38" s="255" t="n"/>
@@ -4918,7 +4943,7 @@
       <c r="AJ39" s="9" t="n"/>
       <c r="AK39" s="21" t="n"/>
       <c r="AM39" s="254">
-        <f>COUNTIF(F39:AL39,"X")</f>
+        <f>COUNTIF(F39:AL39,"A")</f>
         <v/>
       </c>
       <c r="AN39" s="255" t="n"/>
@@ -4967,7 +4992,7 @@
       <c r="AJ40" s="9" t="n"/>
       <c r="AK40" s="21" t="n"/>
       <c r="AM40" s="254">
-        <f>COUNTIF(F40:AL40,"X")</f>
+        <f>COUNTIF(F40:AL40,"A")</f>
         <v/>
       </c>
       <c r="AN40" s="255" t="n"/>
@@ -5016,7 +5041,7 @@
       <c r="AJ41" s="9" t="n"/>
       <c r="AK41" s="21" t="n"/>
       <c r="AM41" s="254">
-        <f>COUNTIF(F41:AL41,"X")</f>
+        <f>COUNTIF(F41:AL41,"A")</f>
         <v/>
       </c>
       <c r="AN41" s="255" t="n"/>
@@ -5065,7 +5090,7 @@
       <c r="AJ42" s="9" t="n"/>
       <c r="AK42" s="21" t="n"/>
       <c r="AM42" s="254">
-        <f>COUNTIF(F42:AL42,"X")</f>
+        <f>COUNTIF(F42:AL42,"A")</f>
         <v/>
       </c>
       <c r="AN42" s="255" t="n"/>
@@ -5114,7 +5139,7 @@
       <c r="AJ43" s="9" t="n"/>
       <c r="AK43" s="21" t="n"/>
       <c r="AM43" s="254">
-        <f>COUNTIF(F43:AL43,"X")</f>
+        <f>COUNTIF(F43:AL43,"A")</f>
         <v/>
       </c>
       <c r="AN43" s="255" t="n"/>
@@ -5163,7 +5188,7 @@
       <c r="AJ44" s="9" t="n"/>
       <c r="AK44" s="21" t="n"/>
       <c r="AM44" s="254">
-        <f>COUNTIF(F44:AL44,"X")</f>
+        <f>COUNTIF(F44:AL44,"A")</f>
         <v/>
       </c>
       <c r="AN44" s="255" t="n"/>
@@ -5212,7 +5237,7 @@
       <c r="AJ45" s="9" t="n"/>
       <c r="AK45" s="21" t="n"/>
       <c r="AM45" s="254">
-        <f>COUNTIF(F45:AL45,"X")</f>
+        <f>COUNTIF(F45:AL45,"A")</f>
         <v/>
       </c>
       <c r="AN45" s="255" t="n"/>
@@ -5263,7 +5288,7 @@
       <c r="AJ46" s="9" t="n"/>
       <c r="AK46" s="179" t="n"/>
       <c r="AM46" s="254">
-        <f>COUNTIF(F46:AL46,"X")</f>
+        <f>COUNTIF(F46:AL46,"A")</f>
         <v/>
       </c>
       <c r="AN46" s="255" t="n"/>
@@ -5314,7 +5339,7 @@
       <c r="AJ47" s="9" t="n"/>
       <c r="AK47" s="179" t="n"/>
       <c r="AM47" s="254">
-        <f>COUNTIF(F47:AL47,"X")</f>
+        <f>COUNTIF(F47:AL47,"A")</f>
         <v/>
       </c>
       <c r="AN47" s="255" t="n"/>
@@ -5365,7 +5390,7 @@
       <c r="AJ48" s="179" t="n"/>
       <c r="AK48" s="179" t="n"/>
       <c r="AM48" s="254">
-        <f>COUNTIF(F48:AL48,"X")</f>
+        <f>COUNTIF(F48:AL48,"A")</f>
         <v/>
       </c>
       <c r="AN48" s="255" t="n"/>
@@ -5416,7 +5441,7 @@
       <c r="AJ49" s="179" t="n"/>
       <c r="AK49" s="179" t="n"/>
       <c r="AM49" s="254">
-        <f>COUNTIF(F49:AL49,"X")</f>
+        <f>COUNTIF(F49:AL49,"A")</f>
         <v/>
       </c>
       <c r="AN49" s="255" t="n"/>
@@ -5467,7 +5492,7 @@
       <c r="AJ50" s="179" t="n"/>
       <c r="AK50" s="179" t="n"/>
       <c r="AM50" s="254">
-        <f>COUNTIF(F50:AL50,"X")</f>
+        <f>COUNTIF(F50:AL50,"A")</f>
         <v/>
       </c>
       <c r="AN50" s="255" t="n"/>
@@ -5516,7 +5541,7 @@
       <c r="AJ51" s="9" t="n"/>
       <c r="AK51" s="21" t="n"/>
       <c r="AM51" s="254">
-        <f>COUNTIF(F51:AL51,"X")</f>
+        <f>COUNTIF(F51:AL51,"A")</f>
         <v/>
       </c>
       <c r="AN51" s="255" t="n"/>
@@ -5565,7 +5590,7 @@
       <c r="AJ52" s="9" t="n"/>
       <c r="AK52" s="21" t="n"/>
       <c r="AM52" s="254">
-        <f>COUNTIF(F52:AL52,"X")</f>
+        <f>COUNTIF(F52:AL52,"A")</f>
         <v/>
       </c>
       <c r="AN52" s="255" t="n"/>
@@ -5614,7 +5639,7 @@
       <c r="AJ53" s="9" t="n"/>
       <c r="AK53" s="21" t="n"/>
       <c r="AM53" s="254">
-        <f>COUNTIF(F53:AL53,"X")</f>
+        <f>COUNTIF(F53:AL53,"A")</f>
         <v/>
       </c>
       <c r="AN53" s="255" t="n"/>
@@ -5663,7 +5688,7 @@
       <c r="AJ54" s="9" t="n"/>
       <c r="AK54" s="21" t="n"/>
       <c r="AM54" s="254">
-        <f>COUNTIF(F54:AL54,"X")</f>
+        <f>COUNTIF(F54:AL54,"A")</f>
         <v/>
       </c>
       <c r="AN54" s="255" t="n"/>
@@ -5714,7 +5739,7 @@
       <c r="AJ55" s="9" t="n"/>
       <c r="AK55" s="179" t="n"/>
       <c r="AM55" s="254">
-        <f>COUNTIF(F55:AL55,"X")</f>
+        <f>COUNTIF(F55:AL55,"A")</f>
         <v/>
       </c>
       <c r="AN55" s="255" t="n"/>
@@ -5765,7 +5790,7 @@
       <c r="AJ56" s="9" t="n"/>
       <c r="AK56" s="179" t="n"/>
       <c r="AM56" s="254">
-        <f>COUNTIF(F56:AL56,"X")</f>
+        <f>COUNTIF(F56:AL56,"A")</f>
         <v/>
       </c>
       <c r="AN56" s="255" t="n"/>
@@ -5816,7 +5841,7 @@
       <c r="AJ57" s="179" t="n"/>
       <c r="AK57" s="179" t="n"/>
       <c r="AM57" s="254">
-        <f>COUNTIF(F57:AL57,"X")</f>
+        <f>COUNTIF(F57:AL57,"A")</f>
         <v/>
       </c>
       <c r="AN57" s="255" t="n"/>
@@ -5866,9 +5891,15 @@
       <c r="AI58" s="22" t="n"/>
       <c r="AJ58" s="179" t="n"/>
       <c r="AK58" s="179" t="n"/>
-      <c r="AM58" s="254" t="n"/>
+      <c r="AM58" s="254">
+        <f>COUNTIF(F58:AL58,"A")</f>
+        <v/>
+      </c>
       <c r="AN58" s="255" t="n"/>
-      <c r="AO58" s="254" t="n"/>
+      <c r="AO58" s="254">
+        <f>AW4-AM58</f>
+        <v/>
+      </c>
       <c r="AP58" s="255" t="n"/>
       <c r="AQ58" s="48" t="n"/>
       <c r="AR58" s="220" t="n"/>
@@ -5911,9 +5942,15 @@
       <c r="AI59" s="22" t="n"/>
       <c r="AJ59" s="179" t="n"/>
       <c r="AK59" s="179" t="n"/>
-      <c r="AM59" s="254" t="n"/>
+      <c r="AM59" s="254">
+        <f>COUNTIF(F59:AL59,"A")</f>
+        <v/>
+      </c>
       <c r="AN59" s="255" t="n"/>
-      <c r="AO59" s="254" t="n"/>
+      <c r="AO59" s="254">
+        <f>AW4-AM59</f>
+        <v/>
+      </c>
       <c r="AP59" s="255" t="n"/>
       <c r="AQ59" s="48" t="n"/>
       <c r="AR59" s="220" t="n"/>
@@ -5954,9 +5991,15 @@
       <c r="AI60" s="38" t="n"/>
       <c r="AJ60" s="9" t="n"/>
       <c r="AK60" s="179" t="n"/>
-      <c r="AM60" s="254" t="n"/>
+      <c r="AM60" s="254">
+        <f>COUNTIF(F60:AL60,"A")</f>
+        <v/>
+      </c>
       <c r="AN60" s="255" t="n"/>
-      <c r="AO60" s="254" t="n"/>
+      <c r="AO60" s="254">
+        <f>AW4-AM60</f>
+        <v/>
+      </c>
       <c r="AP60" s="255" t="n"/>
       <c r="AQ60" s="48" t="n"/>
       <c r="AR60" s="220" t="n"/>
@@ -6093,18 +6136,10 @@
       <c r="AJ63" s="291" t="n"/>
       <c r="AK63" s="242" t="n"/>
       <c r="AL63" s="4" t="n"/>
-      <c r="AM63" s="292" t="inlineStr">
-        <is>
-          <t>Month :              JUNE</t>
-        </is>
-      </c>
+      <c r="AM63" s="292" t="n"/>
       <c r="AN63" s="223" t="n"/>
       <c r="AO63" s="231" t="n"/>
-      <c r="AP63" s="293" t="inlineStr">
-        <is>
-          <t>No. of Days of Classes: 16</t>
-        </is>
-      </c>
+      <c r="AP63" s="293" t="n"/>
       <c r="AQ63" s="231" t="n"/>
       <c r="AR63" s="294" t="inlineStr">
         <is>
@@ -6164,16 +6199,9 @@
         </is>
       </c>
       <c r="AQ65" s="248" t="n"/>
-      <c r="AR65" s="299" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS65" s="300" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT65" s="301">
-        <f>SUM(AR65:AS66)</f>
-        <v/>
-      </c>
+      <c r="AR65" s="299" t="n"/>
+      <c r="AS65" s="300" t="n"/>
+      <c r="AT65" s="301" t="n"/>
       <c r="AU65" s="302" t="n"/>
     </row>
     <row r="66" ht="7.5" customHeight="1" s="204">
@@ -6212,16 +6240,9 @@
         </is>
       </c>
       <c r="AQ67" s="248" t="n"/>
-      <c r="AR67" s="300" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS67" s="300" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT67" s="311">
-        <f>SUM(AR67:AS70)</f>
-        <v/>
-      </c>
+      <c r="AR67" s="300" t="n"/>
+      <c r="AS67" s="300" t="n"/>
+      <c r="AT67" s="311" t="n"/>
       <c r="AU67" s="302" t="n"/>
     </row>
     <row r="68" ht="6.75" customHeight="1" s="204">
@@ -6363,16 +6384,9 @@
       <c r="AO71" s="291" t="n"/>
       <c r="AP71" s="291" t="n"/>
       <c r="AQ71" s="242" t="n"/>
-      <c r="AR71" s="316" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS71" s="316" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT71" s="317">
-        <f>SUM(AR71:AS72)</f>
-        <v/>
-      </c>
+      <c r="AR71" s="316" t="n"/>
+      <c r="AS71" s="316" t="n"/>
+      <c r="AT71" s="317" t="n"/>
       <c r="AU71" s="302" t="n"/>
     </row>
     <row r="72" ht="9.75" customHeight="1" s="204">
@@ -6449,18 +6463,9 @@
       <c r="AO73" s="291" t="n"/>
       <c r="AP73" s="291" t="n"/>
       <c r="AQ73" s="242" t="n"/>
-      <c r="AR73" s="319">
-        <f>(AR71/AR65)*100%</f>
-        <v/>
-      </c>
-      <c r="AS73" s="319">
-        <f>(AS71/AS65)*100%</f>
-        <v/>
-      </c>
-      <c r="AT73" s="320">
-        <f>(AT71/AT65)*100%</f>
-        <v/>
-      </c>
+      <c r="AR73" s="319" t="n"/>
+      <c r="AS73" s="319" t="n"/>
+      <c r="AT73" s="320" t="n"/>
       <c r="AU73" s="302" t="n"/>
     </row>
     <row r="74" ht="12" customHeight="1" s="204">
@@ -6539,18 +6544,9 @@
         </is>
       </c>
       <c r="AQ75" s="248" t="n"/>
-      <c r="AR75" s="17">
-        <f>AO33/AW4*100%%</f>
-        <v/>
-      </c>
-      <c r="AS75" s="17">
-        <f>AO61/AW4*100%%</f>
-        <v/>
-      </c>
-      <c r="AT75" s="321">
-        <f>AO62/AW4*100%%</f>
-        <v/>
-      </c>
+      <c r="AR75" s="17" t="n"/>
+      <c r="AS75" s="17" t="n"/>
+      <c r="AT75" s="321" t="n"/>
       <c r="AU75" s="302" t="n"/>
     </row>
     <row r="76" ht="1.5" customHeight="1" s="204">
@@ -6589,18 +6585,9 @@
       <c r="AO77" s="305" t="n"/>
       <c r="AP77" s="305" t="n"/>
       <c r="AQ77" s="258" t="n"/>
-      <c r="AR77" s="17">
-        <f>AR75/AR71*100</f>
-        <v/>
-      </c>
-      <c r="AS77" s="17">
-        <f>AS75/AS71*100</f>
-        <v/>
-      </c>
-      <c r="AT77" s="321">
-        <f>AT75/AT71*100</f>
-        <v/>
-      </c>
+      <c r="AR77" s="17" t="n"/>
+      <c r="AS77" s="17" t="n"/>
+      <c r="AT77" s="321" t="n"/>
       <c r="AU77" s="255" t="n"/>
     </row>
     <row r="78" ht="17.25" customHeight="1" s="204">
@@ -6617,16 +6604,9 @@
       <c r="AO78" s="305" t="n"/>
       <c r="AP78" s="305" t="n"/>
       <c r="AQ78" s="258" t="n"/>
-      <c r="AR78" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS78" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT78" s="322">
-        <f>SUM(AR78:AS78)</f>
-        <v/>
-      </c>
+      <c r="AR78" s="18" t="n"/>
+      <c r="AS78" s="18" t="n"/>
+      <c r="AT78" s="322" t="n"/>
       <c r="AU78" s="255" t="n"/>
     </row>
     <row r="79" ht="9.75" customHeight="1" s="204">
@@ -6643,16 +6623,9 @@
       <c r="AO79" s="291" t="n"/>
       <c r="AP79" s="291" t="n"/>
       <c r="AQ79" s="242" t="n"/>
-      <c r="AR79" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS79" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT79" s="322">
-        <f>SUM(AR79:AS80)</f>
-        <v/>
-      </c>
+      <c r="AR79" s="18" t="n"/>
+      <c r="AS79" s="18" t="n"/>
+      <c r="AT79" s="322" t="n"/>
       <c r="AU79" s="302" t="n"/>
     </row>
     <row r="80" ht="9.75" customHeight="1" s="204">
@@ -6716,16 +6689,9 @@
         </is>
       </c>
       <c r="AQ81" s="248" t="n"/>
-      <c r="AR81" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS81" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT81" s="322">
-        <f>SUM(AR81:AS82)</f>
-        <v/>
-      </c>
+      <c r="AR81" s="18" t="n"/>
+      <c r="AS81" s="18" t="n"/>
+      <c r="AT81" s="322" t="n"/>
       <c r="AU81" s="302" t="n"/>
     </row>
     <row r="82" ht="9.75" customHeight="1" s="204">
@@ -6787,16 +6753,9 @@
         </is>
       </c>
       <c r="AQ83" s="248" t="n"/>
-      <c r="AR83" s="333" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS83" s="333" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT83" s="322">
-        <f>SUM(AR83:AS84)</f>
-        <v/>
-      </c>
+      <c r="AR83" s="333" t="n"/>
+      <c r="AS83" s="333" t="n"/>
+      <c r="AT83" s="322" t="n"/>
       <c r="AU83" s="302" t="n"/>
     </row>
     <row r="84" ht="15" customHeight="1" s="204" thickBot="1">

</xml_diff>